<commit_message>
July 25 2024- changes -2
</commit_message>
<xml_diff>
--- a/TestData/T2278_TMTI0036294_TMTI0036296_EventExpense_EmailNotification_RequestMoreInformationApproveAsFirstLevelApprover.xlsx
+++ b/TestData/T2278_TMTI0036294_TMTI0036296_EventExpense_EmailNotification_RequestMoreInformationApproveAsFirstLevelApprover.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA461D32-9CB6-45AC-8713-94E7F02DF276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98253CCA-ACC0-4B64-B16C-8D100E5B2B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ExpenseRequest" sheetId="1" r:id="rId1"/>
-    <sheet name="Approver" sheetId="3" r:id="rId2"/>
-    <sheet name="Users" sheetId="2" r:id="rId3"/>
+    <sheet name="Users" sheetId="2" r:id="rId2"/>
+    <sheet name="Approver" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -495,27 +495,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" customWidth="1"/>
-    <col min="8" max="8" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -568,7 +568,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -624,7 +624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -687,15 +687,52 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="1"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -703,7 +740,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>38</v>
       </c>
@@ -714,7 +751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>39</v>
       </c>
@@ -733,41 +770,4 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>